<commit_message>
test: add validation tests for committed XLSX sample and update exception rules
</commit_message>
<xml_diff>
--- a/backend/sample_data/d2c_order_followup_sample_109.xlsx
+++ b/backend/sample_data/d2c_order_followup_sample_109.xlsx
@@ -1,17 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Orders" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Orders" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Orders'!$A$1:$J$110</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -19,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -39,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -47,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,66 +415,54 @@
   </sheetPr>
   <dimension ref="A1:J110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="21" customWidth="1" min="2" max="2"/>
-    <col width="21" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="25" customWidth="1" min="7" max="7"/>
-    <col width="21" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
-    <col width="19" customWidth="1" min="10" max="10"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Order ID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Order date</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Customer name</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Phone</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Order value</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Payment type</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Order status</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Dispatch date</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Expected delivery date</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Assigned employee</t>
         </is>
@@ -515,8 +489,10 @@
           <t>98700000001</t>
         </is>
       </c>
-      <c r="E2" t="n">
-        <v>767</v>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>767</t>
+        </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -565,8 +541,10 @@
           <t>98700000002</t>
         </is>
       </c>
-      <c r="E3" t="n">
-        <v>1084</v>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>1084</t>
+        </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -615,8 +593,10 @@
           <t>98700000003</t>
         </is>
       </c>
-      <c r="E4" t="n">
-        <v>1401</v>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>1401</t>
+        </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -665,8 +645,10 @@
           <t>98700000004</t>
         </is>
       </c>
-      <c r="E5" t="n">
-        <v>1718</v>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>1718</t>
+        </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -715,8 +697,10 @@
           <t>98700000005</t>
         </is>
       </c>
-      <c r="E6" t="n">
-        <v>2035</v>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2035</t>
+        </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -765,8 +749,10 @@
           <t>98700000006</t>
         </is>
       </c>
-      <c r="E7" t="n">
-        <v>2352</v>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2352</t>
+        </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -815,8 +801,10 @@
           <t>98700000007</t>
         </is>
       </c>
-      <c r="E8" t="n">
-        <v>2669</v>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>2669</t>
+        </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -865,8 +853,10 @@
           <t>98700000008</t>
         </is>
       </c>
-      <c r="E9" t="n">
-        <v>2986</v>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2986</t>
+        </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -915,8 +905,10 @@
           <t>98700000009</t>
         </is>
       </c>
-      <c r="E10" t="n">
-        <v>3303</v>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>3303</t>
+        </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -965,8 +957,10 @@
           <t>98700000010</t>
         </is>
       </c>
-      <c r="E11" t="n">
-        <v>3620</v>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>3620</t>
+        </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -1015,8 +1009,10 @@
           <t>98700000011</t>
         </is>
       </c>
-      <c r="E12" t="n">
-        <v>3937</v>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>3937</t>
+        </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -1065,8 +1061,10 @@
           <t>98700000012</t>
         </is>
       </c>
-      <c r="E13" t="n">
-        <v>4254</v>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>4254</t>
+        </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -1115,8 +1113,10 @@
           <t>98700000013</t>
         </is>
       </c>
-      <c r="E14" t="n">
-        <v>4571</v>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>4571</t>
+        </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -1165,8 +1165,10 @@
           <t>98700000014</t>
         </is>
       </c>
-      <c r="E15" t="n">
-        <v>4888</v>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>4888</t>
+        </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -1215,8 +1217,10 @@
           <t>98700000015</t>
         </is>
       </c>
-      <c r="E16" t="n">
-        <v>5205</v>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>5205</t>
+        </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -1265,8 +1269,10 @@
           <t>98700000016</t>
         </is>
       </c>
-      <c r="E17" t="n">
-        <v>5522</v>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>5522</t>
+        </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -1315,8 +1321,10 @@
           <t>98700000017</t>
         </is>
       </c>
-      <c r="E18" t="n">
-        <v>5839</v>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>5839</t>
+        </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -1365,8 +1373,10 @@
           <t>98700000018</t>
         </is>
       </c>
-      <c r="E19" t="n">
-        <v>6156</v>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>6156</t>
+        </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -1415,8 +1425,10 @@
           <t>98700000019</t>
         </is>
       </c>
-      <c r="E20" t="n">
-        <v>6473</v>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>6473</t>
+        </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -1465,8 +1477,10 @@
           <t>98700000020</t>
         </is>
       </c>
-      <c r="E21" t="n">
-        <v>6790</v>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>6790</t>
+        </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -1515,8 +1529,10 @@
           <t>98700000021</t>
         </is>
       </c>
-      <c r="E22" t="n">
-        <v>7107</v>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>7107</t>
+        </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
@@ -1565,8 +1581,10 @@
           <t>98700000022</t>
         </is>
       </c>
-      <c r="E23" t="n">
-        <v>7424</v>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>7424</t>
+        </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -1615,8 +1633,10 @@
           <t>98700000023</t>
         </is>
       </c>
-      <c r="E24" t="n">
-        <v>7741</v>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>7741</t>
+        </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
@@ -1665,8 +1685,10 @@
           <t>98700000024</t>
         </is>
       </c>
-      <c r="E25" t="n">
-        <v>8058</v>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>8058</t>
+        </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -1715,8 +1737,10 @@
           <t>98700000025</t>
         </is>
       </c>
-      <c r="E26" t="n">
-        <v>8375</v>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>8375</t>
+        </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -1765,8 +1789,10 @@
           <t>98700000026</t>
         </is>
       </c>
-      <c r="E27" t="n">
-        <v>8692</v>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>8692</t>
+        </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -1815,8 +1841,10 @@
           <t>98700000027</t>
         </is>
       </c>
-      <c r="E28" t="n">
-        <v>509</v>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>509</t>
+        </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -1865,8 +1893,10 @@
           <t>98700000028</t>
         </is>
       </c>
-      <c r="E29" t="n">
-        <v>826</v>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>826</t>
+        </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
@@ -1915,8 +1945,10 @@
           <t>98700000029</t>
         </is>
       </c>
-      <c r="E30" t="n">
-        <v>1143</v>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>1143</t>
+        </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
@@ -1965,8 +1997,10 @@
           <t>98700000030</t>
         </is>
       </c>
-      <c r="E31" t="n">
-        <v>1460</v>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>1460</t>
+        </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
@@ -2015,8 +2049,10 @@
           <t>98700000031</t>
         </is>
       </c>
-      <c r="E32" t="n">
-        <v>1777</v>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>1777</t>
+        </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
@@ -2065,8 +2101,10 @@
           <t>98700000032</t>
         </is>
       </c>
-      <c r="E33" t="n">
-        <v>2094</v>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>2094</t>
+        </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
@@ -2115,8 +2153,10 @@
           <t>98700000033</t>
         </is>
       </c>
-      <c r="E34" t="n">
-        <v>2411</v>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>2411</t>
+        </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
@@ -2165,8 +2205,10 @@
           <t>98700000034</t>
         </is>
       </c>
-      <c r="E35" t="n">
-        <v>2728</v>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>2728</t>
+        </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
@@ -2215,8 +2257,10 @@
           <t>98700000035</t>
         </is>
       </c>
-      <c r="E36" t="n">
-        <v>3045</v>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>3045</t>
+        </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
@@ -2265,8 +2309,10 @@
           <t>98700000036</t>
         </is>
       </c>
-      <c r="E37" t="n">
-        <v>3362</v>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>3362</t>
+        </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
@@ -2315,8 +2361,10 @@
           <t>98700000037</t>
         </is>
       </c>
-      <c r="E38" t="n">
-        <v>3679</v>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>3679</t>
+        </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
@@ -2365,8 +2413,10 @@
           <t>98700000038</t>
         </is>
       </c>
-      <c r="E39" t="n">
-        <v>3996</v>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>3996</t>
+        </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
@@ -2415,8 +2465,10 @@
           <t>98700000039</t>
         </is>
       </c>
-      <c r="E40" t="n">
-        <v>4313</v>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>4313</t>
+        </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
@@ -2465,8 +2517,10 @@
           <t>98700000040</t>
         </is>
       </c>
-      <c r="E41" t="n">
-        <v>4630</v>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>4630</t>
+        </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
@@ -2515,8 +2569,10 @@
           <t>98700000041</t>
         </is>
       </c>
-      <c r="E42" t="n">
-        <v>4947</v>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>4947</t>
+        </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
@@ -2565,8 +2621,10 @@
           <t>98700000042</t>
         </is>
       </c>
-      <c r="E43" t="n">
-        <v>5264</v>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>5264</t>
+        </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
@@ -2615,8 +2673,10 @@
           <t>98700000043</t>
         </is>
       </c>
-      <c r="E44" t="n">
-        <v>5581</v>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>5581</t>
+        </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
@@ -2665,8 +2725,10 @@
           <t>98700000044</t>
         </is>
       </c>
-      <c r="E45" t="n">
-        <v>5898</v>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>5898</t>
+        </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
@@ -2715,8 +2777,10 @@
           <t>98700000045</t>
         </is>
       </c>
-      <c r="E46" t="n">
-        <v>6215</v>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>6215</t>
+        </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
@@ -2765,8 +2829,10 @@
           <t>98700000046</t>
         </is>
       </c>
-      <c r="E47" t="n">
-        <v>6532</v>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>6532</t>
+        </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
@@ -2815,8 +2881,10 @@
           <t>98700000047</t>
         </is>
       </c>
-      <c r="E48" t="n">
-        <v>6849</v>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>6849</t>
+        </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
@@ -2865,8 +2933,10 @@
           <t>98700000048</t>
         </is>
       </c>
-      <c r="E49" t="n">
-        <v>7166</v>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>7166</t>
+        </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
@@ -2915,8 +2985,10 @@
           <t>98700000049</t>
         </is>
       </c>
-      <c r="E50" t="n">
-        <v>7483</v>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>7483</t>
+        </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
@@ -2965,8 +3037,10 @@
           <t>98700000050</t>
         </is>
       </c>
-      <c r="E51" t="n">
-        <v>7800</v>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>7800</t>
+        </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
@@ -3015,8 +3089,10 @@
           <t>98700000051</t>
         </is>
       </c>
-      <c r="E52" t="n">
-        <v>8117</v>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>8117</t>
+        </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
@@ -3065,8 +3141,10 @@
           <t>98700000052</t>
         </is>
       </c>
-      <c r="E53" t="n">
-        <v>8434</v>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>8434</t>
+        </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
@@ -3115,8 +3193,10 @@
           <t>98700000053</t>
         </is>
       </c>
-      <c r="E54" t="n">
-        <v>8751</v>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>8751</t>
+        </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
@@ -3165,8 +3245,10 @@
           <t>98700000054</t>
         </is>
       </c>
-      <c r="E55" t="n">
-        <v>568</v>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>568</t>
+        </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
@@ -3215,8 +3297,10 @@
           <t>98700000055</t>
         </is>
       </c>
-      <c r="E56" t="n">
-        <v>885</v>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>885</t>
+        </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
@@ -3265,8 +3349,10 @@
           <t>98700000056</t>
         </is>
       </c>
-      <c r="E57" t="n">
-        <v>1202</v>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>1202</t>
+        </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
@@ -3315,8 +3401,10 @@
           <t>98700000057</t>
         </is>
       </c>
-      <c r="E58" t="n">
-        <v>1519</v>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>1519</t>
+        </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
@@ -3365,8 +3453,10 @@
           <t>98700000058</t>
         </is>
       </c>
-      <c r="E59" t="n">
-        <v>1836</v>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>1836</t>
+        </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
@@ -3415,8 +3505,10 @@
           <t>98700000059</t>
         </is>
       </c>
-      <c r="E60" t="n">
-        <v>2153</v>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>2153</t>
+        </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
@@ -3465,8 +3557,10 @@
           <t>98700000060</t>
         </is>
       </c>
-      <c r="E61" t="n">
-        <v>2470</v>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>2470</t>
+        </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
@@ -3515,8 +3609,10 @@
           <t>98700000061</t>
         </is>
       </c>
-      <c r="E62" t="n">
-        <v>2787</v>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>2787</t>
+        </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
@@ -3565,8 +3661,10 @@
           <t>98700000062</t>
         </is>
       </c>
-      <c r="E63" t="n">
-        <v>3104</v>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>3104</t>
+        </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
@@ -3615,8 +3713,10 @@
           <t>98700000063</t>
         </is>
       </c>
-      <c r="E64" t="n">
-        <v>3421</v>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>3421</t>
+        </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
@@ -3665,8 +3765,10 @@
           <t>98700000064</t>
         </is>
       </c>
-      <c r="E65" t="n">
-        <v>3738</v>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>3738</t>
+        </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
@@ -3715,8 +3817,10 @@
           <t>98700000065</t>
         </is>
       </c>
-      <c r="E66" t="n">
-        <v>4055</v>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>4055</t>
+        </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
@@ -3765,8 +3869,10 @@
           <t>98700000066</t>
         </is>
       </c>
-      <c r="E67" t="n">
-        <v>4372</v>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>4372</t>
+        </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
@@ -3815,8 +3921,10 @@
           <t>98700000067</t>
         </is>
       </c>
-      <c r="E68" t="n">
-        <v>4689</v>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>4689</t>
+        </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
@@ -3865,8 +3973,10 @@
           <t>98700000068</t>
         </is>
       </c>
-      <c r="E69" t="n">
-        <v>5006</v>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>5006</t>
+        </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
@@ -3915,8 +4025,10 @@
           <t>98700000069</t>
         </is>
       </c>
-      <c r="E70" t="n">
-        <v>5323</v>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>5323</t>
+        </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
@@ -3965,8 +4077,10 @@
           <t>98700000070</t>
         </is>
       </c>
-      <c r="E71" t="n">
-        <v>5640</v>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>5640</t>
+        </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
@@ -4015,8 +4129,10 @@
           <t>98700000071</t>
         </is>
       </c>
-      <c r="E72" t="n">
-        <v>5957</v>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>5957</t>
+        </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
@@ -4065,8 +4181,10 @@
           <t>98700000072</t>
         </is>
       </c>
-      <c r="E73" t="n">
-        <v>6274</v>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>6274</t>
+        </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
@@ -4115,8 +4233,10 @@
           <t>98700000073</t>
         </is>
       </c>
-      <c r="E74" t="n">
-        <v>6591</v>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>6591</t>
+        </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
@@ -4165,8 +4285,10 @@
           <t>98700000074</t>
         </is>
       </c>
-      <c r="E75" t="n">
-        <v>6908</v>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>6908</t>
+        </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
@@ -4215,8 +4337,10 @@
           <t>98700000075</t>
         </is>
       </c>
-      <c r="E76" t="n">
-        <v>7225</v>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>7225</t>
+        </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
@@ -4265,8 +4389,10 @@
           <t>98700000076</t>
         </is>
       </c>
-      <c r="E77" t="n">
-        <v>7542</v>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>7542</t>
+        </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
@@ -4315,8 +4441,10 @@
           <t>98700000077</t>
         </is>
       </c>
-      <c r="E78" t="n">
-        <v>7859</v>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>7859</t>
+        </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
@@ -4365,8 +4493,10 @@
           <t>98700000078</t>
         </is>
       </c>
-      <c r="E79" t="n">
-        <v>8176</v>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>8176</t>
+        </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
@@ -4415,8 +4545,10 @@
           <t>98700000079</t>
         </is>
       </c>
-      <c r="E80" t="n">
-        <v>8493</v>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>8493</t>
+        </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
@@ -4465,8 +4597,10 @@
           <t>98700000080</t>
         </is>
       </c>
-      <c r="E81" t="n">
-        <v>8810</v>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>8810</t>
+        </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
@@ -4515,8 +4649,10 @@
           <t>98700000081</t>
         </is>
       </c>
-      <c r="E82" t="n">
-        <v>627</v>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>627</t>
+        </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
@@ -4565,8 +4701,10 @@
           <t>98700000082</t>
         </is>
       </c>
-      <c r="E83" t="n">
-        <v>944</v>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>944</t>
+        </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
@@ -4615,8 +4753,10 @@
           <t>98700000083</t>
         </is>
       </c>
-      <c r="E84" t="n">
-        <v>1261</v>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>1261</t>
+        </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
@@ -4665,8 +4805,10 @@
           <t>98700000084</t>
         </is>
       </c>
-      <c r="E85" t="n">
-        <v>1578</v>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>1578</t>
+        </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
@@ -4715,8 +4857,10 @@
           <t>98700000085</t>
         </is>
       </c>
-      <c r="E86" t="n">
-        <v>1895</v>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>1895</t>
+        </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
@@ -4765,8 +4909,10 @@
           <t>98700000086</t>
         </is>
       </c>
-      <c r="E87" t="n">
-        <v>2212</v>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>2212</t>
+        </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
@@ -4815,8 +4961,10 @@
           <t>98700000087</t>
         </is>
       </c>
-      <c r="E88" t="n">
-        <v>2529</v>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>2529</t>
+        </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
@@ -4865,8 +5013,10 @@
           <t>98700000088</t>
         </is>
       </c>
-      <c r="E89" t="n">
-        <v>2846</v>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>2846</t>
+        </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
@@ -4915,8 +5065,10 @@
           <t>98700000089</t>
         </is>
       </c>
-      <c r="E90" t="n">
-        <v>3163</v>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>3163</t>
+        </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
@@ -4965,8 +5117,10 @@
           <t>98700000090</t>
         </is>
       </c>
-      <c r="E91" t="n">
-        <v>3480</v>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>3480</t>
+        </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
@@ -5015,8 +5169,10 @@
           <t>98700000091</t>
         </is>
       </c>
-      <c r="E92" t="n">
-        <v>3797</v>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>3797</t>
+        </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
@@ -5065,8 +5221,10 @@
           <t>98700000092</t>
         </is>
       </c>
-      <c r="E93" t="n">
-        <v>4114</v>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>4114</t>
+        </is>
       </c>
       <c r="F93" t="inlineStr">
         <is>
@@ -5115,8 +5273,10 @@
           <t>98700000093</t>
         </is>
       </c>
-      <c r="E94" t="n">
-        <v>4431</v>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>4431</t>
+        </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
@@ -5165,8 +5325,10 @@
           <t>98700000094</t>
         </is>
       </c>
-      <c r="E95" t="n">
-        <v>4748</v>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>4748</t>
+        </is>
       </c>
       <c r="F95" t="inlineStr">
         <is>
@@ -5215,8 +5377,10 @@
           <t>98700000095</t>
         </is>
       </c>
-      <c r="E96" t="n">
-        <v>5065</v>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>5065</t>
+        </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
@@ -5265,8 +5429,10 @@
           <t>98700000096</t>
         </is>
       </c>
-      <c r="E97" t="n">
-        <v>5382</v>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>5382</t>
+        </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
@@ -5315,8 +5481,10 @@
           <t>98700000097</t>
         </is>
       </c>
-      <c r="E98" t="n">
-        <v>5699</v>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>5699</t>
+        </is>
       </c>
       <c r="F98" t="inlineStr">
         <is>
@@ -5365,8 +5533,10 @@
           <t>98700000098</t>
         </is>
       </c>
-      <c r="E99" t="n">
-        <v>6016</v>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>6016</t>
+        </is>
       </c>
       <c r="F99" t="inlineStr">
         <is>
@@ -5415,8 +5585,10 @@
           <t>98700000099</t>
         </is>
       </c>
-      <c r="E100" t="n">
-        <v>6333</v>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>6333</t>
+        </is>
       </c>
       <c r="F100" t="inlineStr">
         <is>
@@ -5465,8 +5637,10 @@
           <t>98700000100</t>
         </is>
       </c>
-      <c r="E101" t="n">
-        <v>6650</v>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>6650</t>
+        </is>
       </c>
       <c r="F101" t="inlineStr">
         <is>
@@ -5515,8 +5689,10 @@
           <t>9876501001</t>
         </is>
       </c>
-      <c r="E102" t="n">
-        <v>1899</v>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>1899</t>
+        </is>
       </c>
       <c r="F102" t="inlineStr">
         <is>
@@ -5528,7 +5704,11 @@
           <t>Unconfirmed</t>
         </is>
       </c>
-      <c r="H102" t="inlineStr"/>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
       <c r="I102" t="inlineStr">
         <is>
           <t>2026-10-24</t>
@@ -5561,8 +5741,10 @@
           <t>9876501002</t>
         </is>
       </c>
-      <c r="E103" t="n">
-        <v>2499</v>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>2499</t>
+        </is>
       </c>
       <c r="F103" t="inlineStr">
         <is>
@@ -5574,7 +5756,11 @@
           <t>Confirmed</t>
         </is>
       </c>
-      <c r="H103" t="inlineStr"/>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
       <c r="I103" t="inlineStr">
         <is>
           <t>2026-10-23</t>
@@ -5607,8 +5793,10 @@
           <t>9876501003</t>
         </is>
       </c>
-      <c r="E104" t="n">
-        <v>3200</v>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>3200</t>
+        </is>
       </c>
       <c r="F104" t="inlineStr">
         <is>
@@ -5657,8 +5845,10 @@
           <t>9876501004</t>
         </is>
       </c>
-      <c r="E105" t="n">
-        <v>1499</v>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>1499</t>
+        </is>
       </c>
       <c r="F105" t="inlineStr">
         <is>
@@ -5707,8 +5897,10 @@
           <t>9876501005</t>
         </is>
       </c>
-      <c r="E106" t="n">
-        <v>7800</v>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>7800</t>
+        </is>
       </c>
       <c r="F106" t="inlineStr">
         <is>
@@ -5717,7 +5909,7 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>Dispatched</t>
+          <t>Undelivered</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
@@ -5757,8 +5949,10 @@
           <t>9876501006</t>
         </is>
       </c>
-      <c r="E107" t="n">
-        <v>2999</v>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>2999</t>
+        </is>
       </c>
       <c r="F107" t="inlineStr">
         <is>
@@ -5770,7 +5964,11 @@
           <t>Confirmed</t>
         </is>
       </c>
-      <c r="H107" t="inlineStr"/>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
       <c r="I107" t="inlineStr">
         <is>
           <t>2026-10-23</t>
@@ -5803,8 +6001,10 @@
           <t>9876501991</t>
         </is>
       </c>
-      <c r="E108" t="n">
-        <v>999</v>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>999</t>
+        </is>
       </c>
       <c r="F108" t="inlineStr">
         <is>
@@ -5845,8 +6045,10 @@
           <t>9876501992</t>
         </is>
       </c>
-      <c r="E109" t="n">
-        <v>1199</v>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>1199</t>
+        </is>
       </c>
       <c r="F109" t="inlineStr">
         <is>
@@ -5891,8 +6093,10 @@
           <t>9876501993</t>
         </is>
       </c>
-      <c r="E110" t="n">
-        <v>2199</v>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>2199</t>
+        </is>
       </c>
       <c r="F110" t="inlineStr">
         <is>
@@ -5921,7 +6125,6 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J110"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>